<commit_message>
Updated ManageBookings in OfficerController
</commit_message>
<xml_diff>
--- a/Data/ApplicationList.xlsx
+++ b/Data/ApplicationList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\BTOSystem\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C17D0BBA-AAC5-4A6F-B44C-8E807D83067E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5450A1CF-F14E-4606-917C-EE578803A60E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43935" yWindow="915" windowWidth="16200" windowHeight="9315" xr2:uid="{C48FD48A-92B3-4304-9D41-60A342772A21}"/>
+    <workbookView xWindow="50670" yWindow="1890" windowWidth="16200" windowHeight="9315" xr2:uid="{C48FD48A-92B3-4304-9D41-60A342772A21}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,16 +56,16 @@
     <t>ID</t>
   </si>
   <si>
-    <t>TWO</t>
-  </si>
-  <si>
     <t>PENDING</t>
   </si>
   <si>
-    <t>THREE</t>
-  </si>
-  <si>
     <t>SUCCESSFUL</t>
+  </si>
+  <si>
+    <t>TWOROOM</t>
+  </si>
+  <si>
+    <t>THREEROOM</t>
   </si>
 </sst>
 </file>
@@ -440,7 +440,7 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="9.59765625" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
     <col min="4" max="4" width="17.86328125" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" customWidth="1"/>
   </cols>
@@ -473,10 +473,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -493,10 +493,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -513,10 +513,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -533,10 +533,10 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E5">
         <v>4</v>

</xml_diff>